<commit_message>
Added feature to sync postgres tables with records older then specific time and added backdil fix logic
</commit_message>
<xml_diff>
--- a/eastel-report-scripts/reports-pipelines/report-generation-mongo/2-Invoice-Recon/2-Invoice-Recon-daily-checkpoints.xlsx
+++ b/eastel-report-scripts/reports-pipelines/report-generation-mongo/2-Invoice-Recon/2-Invoice-Recon-daily-checkpoints.xlsx
@@ -11958,7 +11958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12079,6 +12079,2921 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-06-16T05:50:31.341762Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>33.35257270000875</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "45863013.27"}</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-01T00:00:00Z"),
+        $lt: ISODate("2026-05-02T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:18:29.835557Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>28.95737550000194</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "45210889.66"}</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-02T00:00:00Z"),
+        $lt: ISODate("2026-05-03T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:18:59.454762Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>33.76051249995362</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "44774447.56"}</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-03T00:00:00Z"),
+        $lt: ISODate("2026-05-04T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:19:33.365259Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>29.01006959995721</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "38561674.67"}</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-04T00:00:00Z"),
+        $lt: ISODate("2026-05-05T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:20:02.530199Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>28.74510840000585</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "40242487.12"}</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-05T00:00:00Z"),
+        $lt: ISODate("2026-05-06T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:20:31.434153Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>31.04104299994651</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "43621357.26"}</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-06T00:00:00Z"),
+        $lt: ISODate("2026-05-07T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:21:02.622473Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>31.69102079991717</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "45117999.91"}</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-07T00:00:00Z"),
+        $lt: ISODate("2026-05-08T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:21:34.466504Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>28.94410210009664</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "48447570.72"}</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-08T00:00:00Z"),
+        $lt: ISODate("2026-05-09T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:22:03.560771Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>29.81094859994482</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "50860396.67"}</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-09T00:00:00Z"),
+        $lt: ISODate("2026-05-10T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:22:33.522430Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>28.61490580008831</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "50688559.05"}</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-10T00:00:00Z"),
+        $lt: ISODate("2026-05-11T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:23:02.284044Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>31.45863080001436</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "47864011.75"}</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-11T00:00:00Z"),
+        $lt: ISODate("2026-05-12T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:23:33.910297Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>27.85971740004607</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "48460326.91"}</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-12T00:00:00Z"),
+        $lt: ISODate("2026-05-13T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:24:01.975119Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>30.59228109999094</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "50307891.47"}</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-13T00:00:00Z"),
+        $lt: ISODate("2026-05-14T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:24:32.717857Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>28.41212639992591</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "50571692.26"}</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-14T00:00:00Z"),
+        $lt: ISODate("2026-05-15T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:25:01.274159Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>30.69236399990041</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "53577032.59"}</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-15T00:00:00Z"),
+        $lt: ISODate("2026-05-16T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:25:32.111295Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>25.50780409993604</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "31574026.54"}</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-16T00:00:00Z"),
+        $lt: ISODate("2026-05-17T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:25:57.846579Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>29.15934420004487</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "523551.96"}</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-17T00:00:00Z"),
+        $lt: ISODate("2026-05-18T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:26:27.201826Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>33.13561320002191</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "496930.23"}</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-18T00:00:00Z"),
+        $lt: ISODate("2026-05-19T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:27:00.567405Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>33.12779219995718</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "422047.02"}</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-19T00:00:00Z"),
+        $lt: ISODate("2026-05-20T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:27:33.866542Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>38.24631010007579</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "395011.18"}</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-20T00:00:00Z"),
+        $lt: ISODate("2026-05-21T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:28:12.267287Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>33.73843270004727</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "447608.26"}</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-21T00:00:00Z"),
+        $lt: ISODate("2026-05-22T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:28:46.155715Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>31.10627099999692</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "435237.53"}</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-22T00:00:00Z"),
+        $lt: ISODate("2026-05-23T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:29:17.408870Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>35.49644659995101</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "522129.00"}</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-23T00:00:00Z"),
+        $lt: ISODate("2026-05-24T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:29:53.037999Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>31.7765756000299</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "490229.31"}</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-24T00:00:00Z"),
+        $lt: ISODate("2026-05-25T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:30:24.958827Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>36.34284890000708</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "523134.98"}</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-25T00:00:00Z"),
+        $lt: ISODate("2026-05-26T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:31:01.468781Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>33.10478449997026</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "624634.39"}</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-26T00:00:00Z"),
+        $lt: ISODate("2026-05-27T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:31:34.704030Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>34.68313020002097</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "485695.65"}</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-27T00:00:00Z"),
+        $lt: ISODate("2026-05-28T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:32:09.525943Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>33.65686700004153</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "518739.45"}</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-28T00:00:00Z"),
+        $lt: ISODate("2026-05-29T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:32:43.400042Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>36.27789259993006</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "715868.15"}</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-29T00:00:00Z"),
+        $lt: ISODate("2026-05-30T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:33:19.915764Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>35.749987600022</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "478815.55"}</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-30T00:00:00Z"),
+        $lt: ISODate("2026-05-31T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:33:55.883136Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>35.82615560002159</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>{"service_type": "Data", "charge_type": "Data MO", "data_type": "4G", "mou_mbs": "434817.56"}</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/*
+Query 6: Domestic 4G data usage in MB.
+Output:
+{
+  service_type: "Data",
+  charge_type: "Data MO",
+  data_type: "4G",
+  mou_mbs: 969335074
+}
+Equivalent PostgreSQL:
+SELECT
+    'Data' AS service_type,
+    'Data MO' AS charge_type,
+    '4G' AS data_type,
+    ROUND(SUM(COALESCE(t.act_update_used_volume, 0)::numeric / 1048576), 2) AS mou_mbs
+FROM iot_portal_tb_request_log t
+WHERE t.req_time &gt;= '2026-04-01'
+  AND t.req_time &lt; '2026-05-01'
+  AND t.rat_type = '4G'
+  AND t.roaming_destination_id = 87
+  AND t.rating_group &lt;&gt; '500003';
+*/
+db.request_logs.aggregate([
+  {
+    $match: {
+      req_time: {
+        $gte: ISODate("2026-05-31T00:00:00Z"),
+        $lt: ISODate("2026-06-01T00:00:00Z")
+      },
+      rat_type: "4G",
+      roaming_destination_id: 87,
+      rating_group: { $nin: ["500003"] }
+    }
+  },
+  {
+    $group: {
+      _id: null,
+      total_bytes: {
+        $sum: {
+          $toDecimal: { $ifNull: ["$act_update_used_volume", 0] }
+        }
+      }
+    }
+  },
+  {
+    $project: {
+      _id: 0,
+      service_type: { $literal: "Data" },
+      charge_type: { $literal: "Data MO" },
+      data_type: { $literal: "4G" },
+      mou_mbs: {
+        $round: [
+          {
+            $divide: [
+              "$total_bytes",
+              { $toDecimal: 1048576 }
+            ]
+          },
+          2
+        ]
+      }
+    }
+  }
+]);
+</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-07-01T10:34:31.893169Z</t>
         </is>
       </c>
     </row>
@@ -12616,7 +15531,6 @@
 </t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-06-19T06:13:27.034025Z</t>

</xml_diff>